<commit_message>
week 1 day 2 stuff!
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B16C32B5-AEDF-5940-A9A5-F44F540BCD22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8794A1FF-C19E-FB41-B227-6117CBA57AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>week</t>
   </si>
@@ -186,6 +186,12 @@
   </si>
   <si>
     <t>reading/week-1.1.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-1/w1-notebooks.qmd</t>
+  </si>
+  <si>
+    <t>labs/lab1/lab1-quarto.qmd</t>
   </si>
 </sst>
 </file>
@@ -579,10 +585,14 @@
       <c r="D3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E3" s="1"/>
+      <c r="E3" s="3" t="s">
+        <v>51</v>
+      </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="H3" s="1" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1">

</xml_diff>

<commit_message>
day 2 notes and slide updates
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8794A1FF-C19E-FB41-B227-6117CBA57AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D457C432-D7CD-C34E-8E19-F3B5CD8969ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>week</t>
   </si>
@@ -192,6 +192,12 @@
   </si>
   <si>
     <t>labs/lab1/lab1-quarto.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-1.2.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w1.2-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -588,10 +594,15 @@
       <c r="E3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F3" s="1"/>
+      <c r="F3" s="3" t="s">
+        <v>54</v>
+      </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
rendered week 2 monday materials
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D457C432-D7CD-C34E-8E19-F3B5CD8969ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D0DB06A-7FEC-354D-8BCB-5935D6EA3F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
week 2 wednesday stuff
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E55F10C6-5E76-2C43-A99F-C3E5E40F05C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{102A6D08-F3AB-A647-A4A4-62DFAB5BD795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21040" yWindow="-19660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-22200" yWindow="-19140" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>week</t>
   </si>
@@ -210,6 +210,15 @@
   </si>
   <si>
     <t>reading/week-2.1.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-2/w2-import-graphics.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w2.2-handout.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-2.2.qmd</t>
   </si>
 </sst>
 </file>
@@ -220,7 +229,7 @@
     <numFmt numFmtId="164" formatCode="mmmm\ d"/>
     <numFmt numFmtId="165" formatCode="mmm\ d"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -233,13 +242,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -293,16 +295,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -566,7 +567,7 @@
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="8">
         <v>46111</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -575,17 +576,16 @@
       <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" t="s">
         <v>49</v>
       </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="3" t="s">
+      <c r="I2" t="s">
         <v>50</v>
       </c>
     </row>
@@ -593,7 +593,7 @@
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <f>B2+2</f>
         <v>46113</v>
       </c>
@@ -603,17 +603,16 @@
       <c r="D3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" t="s">
         <v>51</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" t="s">
         <v>54</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1" t="s">
+      <c r="H3" t="s">
         <v>52</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" t="s">
         <v>53</v>
       </c>
     </row>
@@ -621,7 +620,7 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <f>B2+7</f>
         <v>46118</v>
       </c>
@@ -631,16 +630,16 @@
       <c r="D4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" t="s">
         <v>55</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" t="s">
         <v>56</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" t="s">
         <v>57</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" t="s">
         <v>58</v>
       </c>
     </row>
@@ -648,7 +647,7 @@
       <c r="A5" s="1">
         <v>2</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="8">
         <f>B4+2</f>
         <v>46120</v>
       </c>
@@ -658,15 +657,21 @@
       <c r="D5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="1"/>
+      <c r="E5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I5" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1">
         <v>3</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <f>B4+7</f>
         <v>46125</v>
       </c>
@@ -676,15 +681,12 @@
       <c r="D6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="1">
         <v>3</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <f>B6+2</f>
         <v>46127</v>
       </c>
@@ -694,15 +696,12 @@
       <c r="D7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1">
         <v>4</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="8">
         <f>B6+7</f>
         <v>46132</v>
       </c>
@@ -712,15 +711,12 @@
       <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
     </row>
     <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="1">
         <v>4</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="8">
         <f>B8+2</f>
         <v>46134</v>
       </c>
@@ -730,15 +726,12 @@
       <c r="D9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="1">
         <v>5</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="8">
         <f>B8+7</f>
         <v>46139</v>
       </c>
@@ -748,16 +741,12 @@
       <c r="D10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="1"/>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="1">
         <v>5</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="8">
         <f>B10+2</f>
         <v>46141</v>
       </c>
@@ -767,16 +756,12 @@
       <c r="D11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="1"/>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="1">
         <v>6</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="8">
         <f>B10+7</f>
         <v>46146</v>
       </c>
@@ -786,15 +771,12 @@
       <c r="D12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="1"/>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="1">
         <v>6</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="8">
         <f>B12+2</f>
         <v>46148</v>
       </c>
@@ -804,15 +786,12 @@
       <c r="D13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="1">
         <v>7</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="8">
         <f>B12+7</f>
         <v>46153</v>
       </c>
@@ -822,13 +801,12 @@
       <c r="D14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="1">
         <v>7</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="8">
         <f>B14+2</f>
         <v>46155</v>
       </c>
@@ -838,15 +816,12 @@
       <c r="D15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
     </row>
     <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="1">
         <v>8</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="8">
         <f>B14+7</f>
         <v>46160</v>
       </c>
@@ -856,15 +831,12 @@
       <c r="D16" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
     </row>
     <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="1">
         <v>8</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="8">
         <f>B16+2</f>
         <v>46162</v>
       </c>
@@ -874,16 +846,12 @@
       <c r="D17" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
     </row>
     <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="1">
         <v>9</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <v>46169</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -892,16 +860,12 @@
       <c r="D18" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="1"/>
     </row>
     <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="1">
         <v>10</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="8">
         <f>B18+5</f>
         <v>46174</v>
       </c>
@@ -911,88 +875,85 @@
       <c r="D19" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="3"/>
-      <c r="G19" s="3"/>
     </row>
     <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="1">
         <v>10</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="8">
         <f>B19+2</f>
         <v>46176</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="4" t="s">
         <v>38</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E20" s="3"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E21" s="6"/>
+      <c r="E21" s="5"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E22" s="6"/>
+      <c r="E22" s="5"/>
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E23" s="6"/>
+      <c r="E23" s="5"/>
     </row>
     <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E24" s="6"/>
+      <c r="E24" s="5"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E25" s="6"/>
+      <c r="E25" s="5"/>
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="H26" s="1"/>
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E27" s="6"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E28" s="7"/>
+      <c r="E28" s="6"/>
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E29" s="8"/>
+      <c r="E29" s="7"/>
       <c r="H29" s="1"/>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E30" s="7"/>
+      <c r="E30" s="6"/>
       <c r="H30" s="1"/>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="H31" s="1"/>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E32" s="7"/>
+      <c r="E32" s="6"/>
     </row>
     <row r="33" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E33" s="4"/>
+      <c r="E33" s="3"/>
     </row>
     <row r="34" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E34" s="7"/>
+      <c r="E34" s="6"/>
       <c r="H34" s="1"/>
     </row>
     <row r="35" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E35" s="7"/>
+      <c r="E35" s="6"/>
       <c r="H35" s="1"/>
     </row>
     <row r="36" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E36" s="1"/>
     </row>
     <row r="38" spans="5:8" ht="13" x14ac:dyDescent="0.15">
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
     </row>
     <row r="39" spans="5:8" ht="13" x14ac:dyDescent="0.15">
-      <c r="E39" s="4"/>
+      <c r="E39" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
week 3 day 2 readings and fixing indexing
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE435214-948B-F242-ADE7-8C595A31F2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4302A3E5-26B8-3347-BC7A-4AA64DE75D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-380" yWindow="680" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
   <si>
     <t>week</t>
   </si>
@@ -222,6 +222,18 @@
   </si>
   <si>
     <t>labs/lab2/lab2-ggplot.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-3/w3-dplyr.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-3/w3-more-dplyr-ethics.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-3.1.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-3.2.qmd</t>
   </si>
 </sst>
 </file>
@@ -538,7 +550,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="4" max="4" width="31.6640625" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26.33203125" customWidth="1"/>
     <col min="7" max="7" width="31.33203125" customWidth="1"/>
     <col min="8" max="8" width="27.5" customWidth="1"/>
@@ -695,6 +707,12 @@
       <c r="D6" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="E6" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="1">
@@ -709,6 +727,12 @@
       </c>
       <c r="D7" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
week 3 day 1 materials
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4302A3E5-26B8-3347-BC7A-4AA64DE75D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D97F46-B5BD-EB42-A642-50E8BAC1DC0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>week</t>
   </si>
@@ -234,6 +234,12 @@
   </si>
   <si>
     <t>reading/week-3.2.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/pa3.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w3.1-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -710,6 +716,12 @@
       <c r="E6" s="9" t="s">
         <v>63</v>
       </c>
+      <c r="F6" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>67</v>
+      </c>
       <c r="I6" s="9" t="s">
         <v>65</v>
       </c>

</xml_diff>

<commit_message>
week 3 day 2 handout
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4269029E-D8CC-754F-902A-57AAEB4B082A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F59864A-381B-0248-AD9C-60E553FA4372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
   <si>
     <t>week</t>
   </si>
@@ -243,6 +243,9 @@
   </si>
   <si>
     <t>labs/lab3/lab3-dplyr.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w3.2-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -746,6 +749,9 @@
       <c r="E7" s="9" t="s">
         <v>64</v>
       </c>
+      <c r="F7" s="9" t="s">
+        <v>70</v>
+      </c>
       <c r="H7" s="9" t="s">
         <v>69</v>
       </c>

</xml_diff>

<commit_message>
w4 day 1 class material
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3604FAC-3224-844B-8E35-3852755E4D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDA5D398-0563-F24A-8CA4-A9A83141DB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25080" yWindow="-19460" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21060" yWindow="-20200" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>week</t>
   </si>
@@ -254,10 +254,16 @@
     <t>reading/week-4.2.qmd</t>
   </si>
   <si>
-    <t>labs/lab3/lab4-childcare.qmd</t>
-  </si>
-  <si>
     <t>practice-activities/pa4.qmd</t>
+  </si>
+  <si>
+    <t>labs/lab4/lab4-childcare.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-4/w4-joins-pivots.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w4.1-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -785,8 +791,14 @@
       <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="E8" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>76</v>
+      </c>
       <c r="G8" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>71</v>
@@ -807,7 +819,7 @@
         <v>12</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I9" s="9" t="s">
         <v>72</v>

</xml_diff>

<commit_message>
week 4 day 2 materials
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDA5D398-0563-F24A-8CA4-A9A83141DB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143A1A95-88BE-FB40-8B2A-1816D3CC430E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21060" yWindow="-20200" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>week</t>
   </si>
@@ -264,6 +264,12 @@
   </si>
   <si>
     <t>student-versions/handouts/w4.1-handout.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-4/w4-factors.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w4.2-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -818,6 +824,12 @@
       <c r="D9" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="E9" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>78</v>
+      </c>
       <c r="H9" s="9" t="s">
         <v>74</v>
       </c>

</xml_diff>

<commit_message>
week 5 reading and day 1
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143A1A95-88BE-FB40-8B2A-1816D3CC430E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83558285-9C78-4542-A7CB-D954CA1A1CED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17320" yWindow="-19580" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
   <si>
     <t>week</t>
   </si>
@@ -270,6 +270,18 @@
   </si>
   <si>
     <t>student-versions/handouts/w4.2-handout.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-5.1.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-5.2.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-5/w5-strings.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w5.1-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -851,6 +863,15 @@
       <c r="D10" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="E10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="1">
@@ -865,6 +886,9 @@
       </c>
       <c r="D11" s="1" t="s">
         <v>14</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
dates slides and handout
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD12490-6CCC-174C-8FCC-AE0F0C810DF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0AB3935-73B6-864C-A5FE-C63992E5296C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17320" yWindow="-19580" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
   <si>
     <t>week</t>
   </si>
@@ -288,6 +288,12 @@
   </si>
   <si>
     <t>practice-activities/pa5-2.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-5/w5-dates.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w5.2-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -896,6 +902,12 @@
       <c r="D11" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="E11" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>86</v>
+      </c>
       <c r="G11" s="9" t="s">
         <v>84</v>
       </c>

</xml_diff>

<commit_message>
dates slide updates + schedule
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F8E353-6B37-F040-9AAF-8B13AF367DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9B1D26-947D-3045-B1B3-CEE0BE0EFDD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17320" yWindow="-19580" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
   <si>
     <t>week</t>
   </si>
@@ -303,6 +303,15 @@
   </si>
   <si>
     <t>labs/lab5/lab5-murder.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-6/w6-version-control.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/pa6.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-6.1.qmd</t>
   </si>
 </sst>
 </file>
@@ -941,6 +950,15 @@
       <c r="D12" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="E12" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="1">

</xml_diff>

<commit_message>
reorder later week topics
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9B1D26-947D-3045-B1B3-CEE0BE0EFDD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3983AA1A-BA2E-DF4D-9AA0-C0554F00169C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20480" yWindow="-20380" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -161,21 +161,9 @@
     <t>More Data Visualization!</t>
   </si>
   <si>
-    <t>Iteration</t>
-  </si>
-  <si>
-    <t>Iteration and Simulation</t>
-  </si>
-  <si>
-    <t>Functional Programming</t>
-  </si>
-  <si>
     <t>Statistical Inference</t>
   </si>
   <si>
-    <t>Advanced Graphics</t>
-  </si>
-  <si>
     <t>slides/week-1/w1-intro-r.qmd</t>
   </si>
   <si>
@@ -312,6 +300,18 @@
   </si>
   <si>
     <t>reading/week-6.1.qmd</t>
+  </si>
+  <si>
+    <t>Simulation</t>
+  </si>
+  <si>
+    <t>Iteration + Nice Tables</t>
+  </si>
+  <si>
+    <t>Model Validation and Advanced Graphics</t>
+  </si>
+  <si>
+    <t>TBD</t>
   </si>
 </sst>
 </file>
@@ -678,16 +678,16 @@
         <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="F2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -705,16 +705,16 @@
         <v>40</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -732,16 +732,16 @@
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="I4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -759,16 +759,16 @@
         <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I5" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -786,16 +786,16 @@
         <v>9</v>
       </c>
       <c r="E6" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="F6" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>67</v>
-      </c>
       <c r="I6" s="9" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -813,16 +813,16 @@
         <v>10</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -840,16 +840,16 @@
         <v>11</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -867,16 +867,16 @@
         <v>12</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -894,16 +894,16 @@
         <v>13</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -921,19 +921,19 @@
         <v>14</v>
       </c>
       <c r="E11" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="H11" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="F11" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>89</v>
-      </c>
       <c r="I11" s="9" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -951,13 +951,13 @@
         <v>15</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1002,7 +1002,7 @@
         <v>33</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>17</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1017,7 +1017,7 @@
         <v>34</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1032,7 +1032,7 @@
         <v>35</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1044,10 +1044,10 @@
         <v>46167</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1062,7 +1062,7 @@
         <v>36</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1077,7 +1077,7 @@
         <v>37</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>45</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1092,7 +1092,7 @@
         <v>38</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
midterm what to expect
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3983AA1A-BA2E-DF4D-9AA0-C0554F00169C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8405880F-085D-DA4A-B0BA-0D15ECD2AC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20480" yWindow="-20380" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
   <si>
     <t>week</t>
   </si>
@@ -312,6 +312,9 @@
   </si>
   <si>
     <t>TBD</t>
+  </si>
+  <si>
+    <t>reading/week-6.2.qmd</t>
   </si>
 </sst>
 </file>
@@ -974,6 +977,9 @@
       <c r="D13" s="1" t="s">
         <v>29</v>
       </c>
+      <c r="I13" s="9" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="1">

</xml_diff>

<commit_message>
week 7 day 1 slides and handout
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8405880F-085D-DA4A-B0BA-0D15ECD2AC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E7762E0-74C6-B74F-B67D-8CB4FB6F33AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="96">
   <si>
     <t>week</t>
   </si>
@@ -315,6 +315,12 @@
   </si>
   <si>
     <t>reading/week-6.2.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-7/w7-functions.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w7.1-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -995,6 +1001,12 @@
       <c r="D14" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="E14" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="1">

</xml_diff>

<commit_message>
week 7 day 1 reading
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E7762E0-74C6-B74F-B67D-8CB4FB6F33AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E6B4D4-0C7A-A646-9E28-3809914B6A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
   <si>
     <t>week</t>
   </si>
@@ -321,6 +321,12 @@
   </si>
   <si>
     <t>student-versions/handouts/w7.1-handout.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-7.1.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/pa7.qmd</t>
   </si>
 </sst>
 </file>
@@ -1007,6 +1013,12 @@
       <c r="F14" s="9" t="s">
         <v>95</v>
       </c>
+      <c r="G14" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="1">

</xml_diff>

<commit_message>
week 7 day 2
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E6B4D4-0C7A-A646-9E28-3809914B6A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8577DFE-CE36-C34F-BB6E-E5CB3A7CF3C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
   <si>
     <t>week</t>
   </si>
@@ -327,6 +327,12 @@
   </si>
   <si>
     <t>practice-activities/pa7.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-7/w7-iteration.qmd</t>
+  </si>
+  <si>
+    <t>labs/lab7/lab7-efficiency.qmd</t>
   </si>
 </sst>
 </file>
@@ -1034,6 +1040,12 @@
       <c r="D15" s="1" t="s">
         <v>90</v>
       </c>
+      <c r="E15" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="1">

</xml_diff>

<commit_message>
week 8 day 1 handout
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04CF3079-32BD-D24B-AD48-CE4592C037E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{379A311C-3219-4746-B357-8234B8C4BBB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
   <si>
     <t>week</t>
   </si>
@@ -351,6 +351,9 @@
   </si>
   <si>
     <t>slides/week-8/w8-data-functions.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w8.1-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -1088,6 +1091,9 @@
       <c r="E16" s="9" t="s">
         <v>105</v>
       </c>
+      <c r="F16" s="9" t="s">
+        <v>106</v>
+      </c>
       <c r="G16" s="9" t="s">
         <v>102</v>
       </c>

</xml_diff>

<commit_message>
fill out week 8
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{379A311C-3219-4746-B357-8234B8C4BBB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA1EF116-027E-C643-BBE7-222A686E180B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="110">
   <si>
     <t>week</t>
   </si>
@@ -347,13 +347,22 @@
     <t>reading/week-8.1.qmd</t>
   </si>
   <si>
-    <t>labs/lab8/lab8-datafunctions.qmd</t>
-  </si>
-  <si>
     <t>slides/week-8/w8-data-functions.qmd</t>
   </si>
   <si>
     <t>student-versions/handouts/w8.1-handout.qmd</t>
+  </si>
+  <si>
+    <t>slides/week-8/w8-simulation.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/pa8-2.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-8.2.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w8.2-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -1089,10 +1098,10 @@
         <v>17</v>
       </c>
       <c r="E16" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="F16" s="9" t="s">
         <v>105</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>106</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>102</v>
@@ -1101,7 +1110,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="1">
         <v>8</v>
       </c>
@@ -1115,11 +1124,23 @@
       <c r="D17" s="1" t="s">
         <v>89</v>
       </c>
+      <c r="E17" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>107</v>
+      </c>
       <c r="H17" s="9" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>102</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="1">
         <v>9</v>
       </c>
@@ -1134,7 +1155,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="1">
         <v>9</v>
       </c>
@@ -1149,7 +1170,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="1">
         <v>10</v>
       </c>
@@ -1164,7 +1185,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="1">
         <v>10</v>
       </c>
@@ -1179,43 +1200,43 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E22" s="5"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
     </row>
-    <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E23" s="5"/>
     </row>
-    <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E24" s="5"/>
     </row>
-    <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E25" s="5"/>
     </row>
-    <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E26" s="5"/>
     </row>
-    <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="H27" s="1"/>
     </row>
-    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E28" s="5"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
     </row>
-    <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E29" s="6"/>
     </row>
-    <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E30" s="7"/>
       <c r="H30" s="1"/>
     </row>
-    <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E31" s="6"/>
       <c r="H31" s="1"/>
     </row>
-    <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="H32" s="1"/>
     </row>
     <row r="33" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
week 9 slides and reading
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BFA4601-6E9E-6A4E-A1FB-AB2C83433274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F918E244-81E4-FA48-8F89-49B9005B545D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17580" yWindow="-20440" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
   <si>
     <t>week</t>
   </si>
@@ -161,9 +161,6 @@
     <t>More Data Visualization!</t>
   </si>
   <si>
-    <t>Statistical Inference</t>
-  </si>
-  <si>
     <t>slides/week-1/w1-intro-r.qmd</t>
   </si>
   <si>
@@ -366,6 +363,15 @@
   </si>
   <si>
     <t>labs/lab8/lab8-datafunctions.qmd</t>
+  </si>
+  <si>
+    <t>Linear Regression</t>
+  </si>
+  <si>
+    <t>slides/week-9/w9-regression.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-9.qmd</t>
   </si>
 </sst>
 </file>
@@ -732,16 +738,16 @@
         <v>7</v>
       </c>
       <c r="E2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" t="s">
         <v>43</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>44</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>45</v>
-      </c>
-      <c r="I2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -759,16 +765,16 @@
         <v>40</v>
       </c>
       <c r="E3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3" t="s">
         <v>47</v>
       </c>
-      <c r="F3" t="s">
-        <v>50</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>48</v>
-      </c>
-      <c r="I3" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -786,16 +792,16 @@
         <v>8</v>
       </c>
       <c r="E4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" t="s">
         <v>51</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>52</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
         <v>53</v>
-      </c>
-      <c r="I4" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -813,16 +819,16 @@
         <v>41</v>
       </c>
       <c r="E5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F5" t="s">
         <v>55</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I5" t="s">
         <v>56</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="I5" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -840,16 +846,16 @@
         <v>9</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -867,16 +873,16 @@
         <v>10</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -894,16 +900,16 @@
         <v>11</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>72</v>
-      </c>
       <c r="G8" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -921,16 +927,16 @@
         <v>12</v>
       </c>
       <c r="E9" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>74</v>
-      </c>
       <c r="H9" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -948,16 +954,16 @@
         <v>13</v>
       </c>
       <c r="E10" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="G10" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="G10" s="9" t="s">
-        <v>79</v>
-      </c>
       <c r="I10" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -975,19 +981,19 @@
         <v>14</v>
       </c>
       <c r="E11" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="F11" s="9" t="s">
-        <v>82</v>
-      </c>
       <c r="G11" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1005,13 +1011,13 @@
         <v>15</v>
       </c>
       <c r="E12" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G12" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="I12" s="9" t="s">
         <v>87</v>
-      </c>
-      <c r="I12" s="9" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1029,7 +1035,7 @@
         <v>29</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1047,16 +1053,16 @@
         <v>16</v>
       </c>
       <c r="E14" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="F14" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="G14" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="I14" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1071,19 +1077,19 @@
         <v>33</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E15" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="H15" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="F15" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="H15" s="9" t="s">
+      <c r="I15" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="I15" s="9" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1101,16 +1107,16 @@
         <v>17</v>
       </c>
       <c r="E16" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="F16" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="F16" s="9" t="s">
-        <v>105</v>
-      </c>
       <c r="G16" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="I16" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="I16" s="9" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1125,22 +1131,22 @@
         <v>35</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E17" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G17" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="H17" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="I17" s="9" t="s">
         <v>107</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1152,10 +1158,10 @@
         <v>46167</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1170,7 +1176,13 @@
         <v>36</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>42</v>
+        <v>110</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1185,7 +1197,7 @@
         <v>37</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1200,7 +1212,7 @@
         <v>38</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
lab 9 fix and lab 9 handout
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F918E244-81E4-FA48-8F89-49B9005B545D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E80EAF2C-6AC2-1C4A-9C45-89CF1E7533DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17580" yWindow="-20440" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="116">
   <si>
     <t>week</t>
   </si>
@@ -372,6 +372,15 @@
   </si>
   <si>
     <t>reading/week-9.qmd</t>
+  </si>
+  <si>
+    <t>student-versions/handouts/w9-handout.qmd</t>
+  </si>
+  <si>
+    <t>labs/lab9/lab9-regression.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-10.qmd</t>
   </si>
 </sst>
 </file>
@@ -1181,6 +1190,12 @@
       <c r="E19" s="9" t="s">
         <v>111</v>
       </c>
+      <c r="F19" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>114</v>
+      </c>
       <c r="I19" s="9" t="s">
         <v>112</v>
       </c>
@@ -1198,6 +1213,9 @@
       </c>
       <c r="D20" s="1" t="s">
         <v>90</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
add wednesday materials to index
</commit_message>
<xml_diff>
--- a/stat-331-s26-schedule.xlsx
+++ b/stat-331-s26-schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat331/stat331-calpoly-s26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D696EAF-BC09-584E-A208-0D567A0ED82B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD2A774-CBBE-0440-B5B8-DA30B0B80622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18860" yWindow="-19580" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
   <si>
     <t>week</t>
   </si>
@@ -308,9 +308,6 @@
     <t>Model Validation and Advanced Graphics</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>reading/week-6.2.qmd</t>
   </si>
   <si>
@@ -390,6 +387,12 @@
   </si>
   <si>
     <t>practice-activities/pa10.qmd</t>
+  </si>
+  <si>
+    <t>Course Review</t>
+  </si>
+  <si>
+    <t>slides/week-10/w10-wrapup.qmd</t>
   </si>
 </sst>
 </file>
@@ -1053,7 +1056,7 @@
         <v>29</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1071,16 +1074,16 @@
         <v>16</v>
       </c>
       <c r="E14" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F14" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="G14" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="I14" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1098,16 +1101,16 @@
         <v>89</v>
       </c>
       <c r="E15" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="H15" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="F15" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="H15" s="9" t="s">
+      <c r="I15" s="9" t="s">
         <v>98</v>
-      </c>
-      <c r="I15" s="9" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1125,16 +1128,16 @@
         <v>17</v>
       </c>
       <c r="E16" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="F16" s="9" t="s">
-        <v>104</v>
-      </c>
       <c r="G16" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="I16" s="9" t="s">
         <v>101</v>
-      </c>
-      <c r="I16" s="9" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1152,19 +1155,19 @@
         <v>88</v>
       </c>
       <c r="E17" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="G17" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="H17" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="I17" s="9" t="s">
         <v>106</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1194,19 +1197,19 @@
         <v>36</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="F19" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="I19" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="H19" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="I19" s="9" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1224,16 +1227,16 @@
         <v>90</v>
       </c>
       <c r="E20" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="F20" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="G20" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="G20" s="9" t="s">
-        <v>118</v>
-      </c>
       <c r="I20" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1248,7 +1251,10 @@
         <v>38</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>91</v>
+        <v>118</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>